<commit_message>
further improvement of shiny rmarkdown workflow
</commit_message>
<xml_diff>
--- a/vdata _DxI.xlsx
+++ b/vdata _DxI.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13130" windowHeight="6110"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="9" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="78">
   <si>
     <t>Projekt</t>
   </si>
@@ -224,49 +224,43 @@
     <t>Julien</t>
   </si>
   <si>
+    <t>stud BMLA</t>
+  </si>
+  <si>
+    <t>Jelena</t>
+  </si>
+  <si>
+    <t>Oliver</t>
+  </si>
+  <si>
+    <t>Mai - Juli 2024</t>
+  </si>
+  <si>
     <t>DxI800</t>
   </si>
   <si>
-    <t>stud BMLA</t>
-  </si>
-  <si>
-    <t>Jelena</t>
-  </si>
-  <si>
-    <t>Oliver</t>
-  </si>
-  <si>
-    <t>Mai - Juli 2024</t>
-  </si>
-  <si>
-    <t>DxI800</t>
-  </si>
-  <si>
     <t>DxI9000</t>
   </si>
   <si>
     <t>Bezeichnung</t>
   </si>
   <si>
+    <t>Methode</t>
+  </si>
+  <si>
     <t>EINHEIT</t>
   </si>
   <si>
     <t>DoseUnit</t>
   </si>
   <si>
-    <t>TSH (3.IS)</t>
-  </si>
-  <si>
-    <t>mlU/l</t>
-  </si>
-  <si>
-    <t>µIU/mL</t>
-  </si>
-  <si>
-    <t>TSH 800</t>
-  </si>
-  <si>
-    <t>TSH 9000</t>
+    <t>Ferritin</t>
+  </si>
+  <si>
+    <t>µg/dl</t>
+  </si>
+  <si>
+    <t>ng/mL</t>
   </si>
 </sst>
 </file>
@@ -289,38 +283,32 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="0" tint="-0.34998626667073579"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -478,50 +466,50 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -536,15 +524,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -557,25 +545,25 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1237,202 +1225,205 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="26.140625" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" customWidth="1"/>
+    <col min="2" max="2" width="26.1796875" customWidth="1"/>
+    <col min="3" max="3" width="30.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="B1" s="17" t="str">
+        <f>DATA!C2</f>
+        <v>Ferritin</v>
+      </c>
+      <c r="C1" s="19" t="str">
+        <f>DATA!C2</f>
+        <v>Ferritin</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="5" t="str">
-        <f>DATA!D2</f>
-        <v>mlU/l</v>
-      </c>
-      <c r="C2" s="5" t="str">
+      <c r="B2" s="2" t="str">
         <f>DATA!E2</f>
-        <v>µIU/mL</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+        <v>µg/dl</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <f>DATA!F2</f>
+        <v>ng/mL</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="3" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="20" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="B6" s="2"/>
+      <c r="C6" s="20"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="7" t="str">
+      <c r="B7" s="21" t="str">
+        <f>DATA!A1</f>
+        <v>DxI800</v>
+      </c>
+      <c r="C7" s="3" t="str">
         <f>DATA!B1</f>
         <v>DxI9000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="6"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+      <c r="B8" s="6"/>
+      <c r="C8" s="20"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="13"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="20" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="10"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="10"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="B11" s="8"/>
+      <c r="C11" s="5"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="20" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C14" s="20" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="5" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="21"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C16" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="7"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="18" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="7"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="B17" s="9"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="6"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
+      <c r="B18" s="11"/>
+      <c r="C18" s="20"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="7"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="B19" s="12"/>
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="6"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="B20" s="11"/>
+      <c r="C20" s="20"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="7"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1443,18 +1434,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" customWidth="1"/>
-    <col min="4" max="5" width="14.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="14.26953125" customWidth="1"/>
+    <col min="4" max="5" width="14.7265625" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" customWidth="1"/>
-    <col min="9" max="9" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.54296875" customWidth="1"/>
+    <col min="9" max="9" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -1483,7 +1474,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="22">
         <v>20</v>
       </c>
@@ -1525,23 +1516,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L73"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="17.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="17.140625" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" customWidth="1"/>
-    <col min="8" max="8" width="17.140625" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" customWidth="1"/>
-    <col min="11" max="11" width="17.140625" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" customWidth="1"/>
+    <col min="2" max="2" width="17.1796875" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" customWidth="1"/>
+    <col min="4" max="4" width="16.7265625" customWidth="1"/>
+    <col min="5" max="5" width="17.1796875" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" customWidth="1"/>
+    <col min="10" max="10" width="14.54296875" customWidth="1"/>
+    <col min="11" max="11" width="17.1796875" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="37" t="s">
         <v>28</v>
       </c>
@@ -1579,7 +1570,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="45" t="s">
         <v>61</v>
       </c>
@@ -1601,7 +1592,7 @@
       <c r="K2" s="44"/>
       <c r="L2" s="46"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="45" t="s">
         <v>61</v>
       </c>
@@ -1623,7 +1614,7 @@
       <c r="K3" s="44"/>
       <c r="L3" s="46"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="45" t="s">
         <v>61</v>
       </c>
@@ -1645,7 +1636,7 @@
       <c r="K4" s="44"/>
       <c r="L4" s="46"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="45" t="s">
         <v>61</v>
       </c>
@@ -1667,7 +1658,7 @@
       <c r="K5" s="44"/>
       <c r="L5" s="46"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="45" t="s">
         <v>61</v>
       </c>
@@ -1689,7 +1680,7 @@
       <c r="K6" s="44"/>
       <c r="L6" s="46"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="45" t="s">
         <v>61</v>
       </c>
@@ -1711,7 +1702,7 @@
       <c r="K7" s="44"/>
       <c r="L7" s="46"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="45" t="s">
         <v>61</v>
       </c>
@@ -1733,7 +1724,7 @@
       <c r="K8" s="44"/>
       <c r="L8" s="46"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="45" t="s">
         <v>61</v>
       </c>
@@ -1755,7 +1746,7 @@
       <c r="K9" s="44"/>
       <c r="L9" s="46"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="45" t="s">
         <v>61</v>
       </c>
@@ -1777,7 +1768,7 @@
       <c r="K10" s="44"/>
       <c r="L10" s="46"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="45" t="s">
         <v>61</v>
       </c>
@@ -1799,12 +1790,12 @@
       <c r="K11" s="44"/>
       <c r="L11" s="46"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="D23" s="52"/>
       <c r="E23" s="52"/>
       <c r="F23" s="52"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="23"/>
       <c r="B24" s="51"/>
       <c r="C24" s="51"/>
@@ -1812,7 +1803,7 @@
       <c r="E24" s="52"/>
       <c r="F24" s="52"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="53"/>
       <c r="B25" s="23"/>
       <c r="C25" s="23"/>
@@ -1820,7 +1811,7 @@
       <c r="E25" s="52"/>
       <c r="F25" s="52"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="30"/>
       <c r="B26" s="31"/>
       <c r="C26" s="31"/>
@@ -1828,7 +1819,7 @@
       <c r="E26" s="30"/>
       <c r="F26" s="31"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="32"/>
       <c r="B27" s="32"/>
       <c r="C27" s="32"/>
@@ -1836,7 +1827,7 @@
       <c r="E27" s="32"/>
       <c r="F27" s="32"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="35"/>
       <c r="B28" s="27"/>
       <c r="C28" s="27"/>
@@ -1844,7 +1835,7 @@
       <c r="E28" s="34"/>
       <c r="F28" s="27"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="33"/>
       <c r="B29" s="27"/>
       <c r="C29" s="27"/>
@@ -1852,7 +1843,7 @@
       <c r="E29" s="33"/>
       <c r="F29" s="27"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="33"/>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -1860,7 +1851,7 @@
       <c r="E30" s="33"/>
       <c r="F30" s="27"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="33"/>
       <c r="B31" s="27"/>
       <c r="C31" s="27"/>
@@ -1868,7 +1859,7 @@
       <c r="E31" s="33"/>
       <c r="F31" s="27"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="33"/>
       <c r="B32" s="27"/>
       <c r="C32" s="27"/>
@@ -1876,7 +1867,7 @@
       <c r="E32" s="33"/>
       <c r="F32" s="27"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="33"/>
       <c r="B33" s="27"/>
       <c r="C33" s="27"/>
@@ -1884,7 +1875,7 @@
       <c r="E33" s="33"/>
       <c r="F33" s="27"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="33"/>
       <c r="B34" s="27"/>
       <c r="C34" s="27"/>
@@ -1892,7 +1883,7 @@
       <c r="E34" s="33"/>
       <c r="F34" s="27"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="33"/>
       <c r="B35" s="27"/>
       <c r="C35" s="27"/>
@@ -1900,7 +1891,7 @@
       <c r="E35" s="33"/>
       <c r="F35" s="27"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="33"/>
       <c r="B36" s="27"/>
       <c r="C36" s="27"/>
@@ -1908,7 +1899,7 @@
       <c r="E36" s="33"/>
       <c r="F36" s="27"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="33"/>
       <c r="B37" s="27"/>
       <c r="C37" s="27"/>
@@ -1916,7 +1907,7 @@
       <c r="E37" s="33"/>
       <c r="F37" s="27"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="36"/>
       <c r="B38" s="25"/>
       <c r="C38" s="25"/>
@@ -1924,7 +1915,7 @@
       <c r="E38" s="61"/>
       <c r="F38" s="25"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="36"/>
       <c r="B39" s="25"/>
       <c r="C39" s="25"/>
@@ -1932,7 +1923,7 @@
       <c r="E39" s="61"/>
       <c r="F39" s="25"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="36"/>
       <c r="B40" s="26"/>
       <c r="C40" s="26"/>
@@ -1940,7 +1931,7 @@
       <c r="E40" s="61"/>
       <c r="F40" s="26"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="49"/>
       <c r="B41" s="49"/>
       <c r="C41" s="49"/>
@@ -1948,7 +1939,7 @@
       <c r="E41" s="49"/>
       <c r="F41" s="49"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="29"/>
       <c r="B42" s="29"/>
       <c r="C42" s="29"/>
@@ -1956,7 +1947,7 @@
       <c r="E42" s="29"/>
       <c r="F42" s="29"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="23"/>
       <c r="B46" s="54"/>
       <c r="C46" s="54"/>
@@ -1964,7 +1955,7 @@
       <c r="E46" s="52"/>
       <c r="F46" s="52"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="23"/>
       <c r="B47" s="54"/>
       <c r="C47" s="54"/>
@@ -1972,7 +1963,7 @@
       <c r="E47" s="52"/>
       <c r="F47" s="52"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="23"/>
       <c r="B48" s="54"/>
       <c r="C48" s="54"/>
@@ -1980,7 +1971,7 @@
       <c r="E48" s="52"/>
       <c r="F48" s="52"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="23"/>
       <c r="B49" s="54"/>
       <c r="C49" s="54"/>
@@ -1988,7 +1979,7 @@
       <c r="E49" s="52"/>
       <c r="F49" s="52"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="23"/>
       <c r="B50" s="54"/>
       <c r="C50" s="54"/>
@@ -1996,7 +1987,7 @@
       <c r="E50" s="52"/>
       <c r="F50" s="52"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="23"/>
       <c r="B51" s="54"/>
       <c r="C51" s="54"/>
@@ -2004,7 +1995,7 @@
       <c r="E51" s="52"/>
       <c r="F51" s="52"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="23"/>
       <c r="B52" s="54"/>
       <c r="C52" s="54"/>
@@ -2012,7 +2003,7 @@
       <c r="E52" s="52"/>
       <c r="F52" s="52"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="23"/>
       <c r="B53" s="54"/>
       <c r="C53" s="54"/>
@@ -2020,7 +2011,7 @@
       <c r="E53" s="52"/>
       <c r="F53" s="52"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="23"/>
       <c r="B54" s="54"/>
       <c r="C54" s="54"/>
@@ -2028,7 +2019,7 @@
       <c r="E54" s="52"/>
       <c r="F54" s="52"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="23"/>
       <c r="B55" s="54"/>
       <c r="C55" s="54"/>
@@ -2036,7 +2027,7 @@
       <c r="E55" s="52"/>
       <c r="F55" s="52"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="23"/>
       <c r="B56" s="24"/>
       <c r="C56" s="24"/>
@@ -2044,7 +2035,7 @@
       <c r="E56" s="52"/>
       <c r="F56" s="52"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="23"/>
       <c r="B57" s="24"/>
       <c r="C57" s="24"/>
@@ -2052,7 +2043,7 @@
       <c r="E57" s="52"/>
       <c r="F57" s="52"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="23"/>
       <c r="B58" s="24"/>
       <c r="C58" s="24"/>
@@ -2060,7 +2051,7 @@
       <c r="E58" s="52"/>
       <c r="F58" s="52"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="23"/>
       <c r="B59" s="24"/>
       <c r="C59" s="24"/>
@@ -2068,7 +2059,7 @@
       <c r="E59" s="52"/>
       <c r="F59" s="52"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="23"/>
       <c r="B60" s="24"/>
       <c r="C60" s="24"/>
@@ -2076,7 +2067,7 @@
       <c r="E60" s="52"/>
       <c r="F60" s="52"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="23"/>
       <c r="B61" s="24"/>
       <c r="C61" s="24"/>
@@ -2084,7 +2075,7 @@
       <c r="E61" s="52"/>
       <c r="F61" s="52"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="23"/>
       <c r="B62" s="24"/>
       <c r="C62" s="24"/>
@@ -2092,7 +2083,7 @@
       <c r="E62" s="52"/>
       <c r="F62" s="52"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="23"/>
       <c r="B63" s="24"/>
       <c r="C63" s="24"/>
@@ -2100,7 +2091,7 @@
       <c r="E63" s="52"/>
       <c r="F63" s="52"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="23"/>
       <c r="B64" s="52"/>
       <c r="C64" s="52"/>
@@ -2108,7 +2099,7 @@
       <c r="E64" s="52"/>
       <c r="F64" s="52"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="23"/>
       <c r="B65" s="52"/>
       <c r="C65" s="52"/>
@@ -2116,7 +2107,7 @@
       <c r="E65" s="52"/>
       <c r="F65" s="52"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="23"/>
       <c r="B66" s="52"/>
       <c r="C66" s="52"/>
@@ -2124,7 +2115,7 @@
       <c r="E66" s="52"/>
       <c r="F66" s="52"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="23"/>
       <c r="B67" s="52"/>
       <c r="C67" s="52"/>
@@ -2132,7 +2123,7 @@
       <c r="E67" s="52"/>
       <c r="F67" s="52"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="23"/>
       <c r="B68" s="52"/>
       <c r="C68" s="52"/>
@@ -2140,7 +2131,7 @@
       <c r="E68" s="52"/>
       <c r="F68" s="52"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="23"/>
       <c r="B69" s="52"/>
       <c r="C69" s="52"/>
@@ -2148,7 +2139,7 @@
       <c r="E69" s="52"/>
       <c r="F69" s="52"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="23"/>
       <c r="B70" s="52"/>
       <c r="C70" s="52"/>
@@ -2156,7 +2147,7 @@
       <c r="E70" s="52"/>
       <c r="F70" s="52"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="23"/>
       <c r="B71" s="52"/>
       <c r="C71" s="52"/>
@@ -2164,7 +2155,7 @@
       <c r="E71" s="52"/>
       <c r="F71" s="52"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="23"/>
       <c r="B72" s="52"/>
       <c r="C72" s="52"/>
@@ -2172,7 +2163,7 @@
       <c r="E72" s="52"/>
       <c r="F72" s="52"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="23"/>
       <c r="B73" s="52"/>
       <c r="C73" s="52"/>
@@ -2197,862 +2188,1383 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E148"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F148"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="17.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="27" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="C1" t="s">
         <v>71</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>73</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="58">
-        <v>1.39</v>
+        <v>36</v>
       </c>
       <c r="B2" s="59">
-        <v>1.6519999999999999</v>
+        <v>30.6</v>
       </c>
       <c r="C2" t="s">
         <v>75</v>
       </c>
-      <c r="D2" t="s">
-        <v>76</v>
+      <c r="D2">
+        <v>37274</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="56">
-        <v>1.47</v>
+        <v>62</v>
       </c>
       <c r="B3" s="57">
-        <v>1.5660000000000001</v>
+        <v>65.3</v>
       </c>
       <c r="C3" t="s">
         <v>75</v>
       </c>
-      <c r="D3" t="s">
-        <v>76</v>
+      <c r="D3">
+        <v>37274</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="58">
-        <v>2.8</v>
+        <v>159</v>
       </c>
       <c r="B4" s="59">
-        <v>3.2719999999999998</v>
+        <v>157.80000000000001</v>
       </c>
       <c r="C4" t="s">
         <v>75</v>
       </c>
-      <c r="D4" t="s">
-        <v>76</v>
+      <c r="D4">
+        <v>37274</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="56">
-        <v>1.91</v>
+        <v>159</v>
       </c>
       <c r="B5" s="57">
-        <v>2.0960000000000001</v>
+        <v>230.6</v>
       </c>
       <c r="C5" t="s">
         <v>75</v>
       </c>
-      <c r="D5" t="s">
-        <v>76</v>
+      <c r="D5">
+        <v>37274</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="58">
-        <v>3.11</v>
+        <v>191</v>
       </c>
       <c r="B6" s="57">
-        <v>3.5939999999999999</v>
+        <v>176.3</v>
       </c>
       <c r="C6" t="s">
         <v>75</v>
       </c>
-      <c r="D6" t="s">
-        <v>76</v>
+      <c r="D6">
+        <v>37274</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="58">
-        <v>0.96399999999999997</v>
+        <v>48</v>
       </c>
       <c r="B7" s="57">
-        <v>1.109</v>
+        <v>43.3</v>
       </c>
       <c r="C7" t="s">
         <v>75</v>
       </c>
-      <c r="D7" t="s">
-        <v>76</v>
+      <c r="D7">
+        <v>37274</v>
       </c>
       <c r="E7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="56">
-        <v>1.59</v>
+        <v>18</v>
       </c>
       <c r="B8" s="59">
-        <v>1.8360000000000001</v>
+        <v>17.2</v>
       </c>
       <c r="C8" t="s">
         <v>75</v>
       </c>
-      <c r="D8" t="s">
-        <v>76</v>
+      <c r="D8">
+        <v>37274</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="58">
-        <v>2.2999999999999998</v>
+        <v>154</v>
       </c>
       <c r="B9" s="57">
-        <v>2.504</v>
+        <v>152.4</v>
       </c>
       <c r="C9" t="s">
         <v>75</v>
       </c>
-      <c r="D9" t="s">
-        <v>76</v>
+      <c r="D9">
+        <v>37274</v>
       </c>
       <c r="E9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="56">
-        <v>0.82099999999999995</v>
+        <v>25</v>
       </c>
       <c r="B10" s="59">
-        <v>1.0309999999999999</v>
+        <v>21.3</v>
       </c>
       <c r="C10" t="s">
         <v>75</v>
       </c>
-      <c r="D10" t="s">
-        <v>76</v>
+      <c r="D10">
+        <v>37274</v>
       </c>
       <c r="E10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="58">
-        <v>3.87</v>
+        <v>45</v>
       </c>
       <c r="B11" s="57">
-        <v>4.5750000000000002</v>
+        <v>42.3</v>
       </c>
       <c r="C11" t="s">
         <v>75</v>
       </c>
-      <c r="D11" t="s">
-        <v>76</v>
+      <c r="D11">
+        <v>37274</v>
       </c>
       <c r="E11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="56">
-        <v>1.37</v>
+        <v>64</v>
       </c>
       <c r="B12" s="59">
-        <v>1.6140000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="C12" t="s">
         <v>75</v>
       </c>
-      <c r="D12" t="s">
-        <v>76</v>
+      <c r="D12">
+        <v>37274</v>
       </c>
       <c r="E12" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="58">
-        <v>2.82</v>
+        <v>64</v>
       </c>
       <c r="B13" s="57">
-        <v>3.266</v>
+        <v>71.2</v>
       </c>
       <c r="C13" t="s">
         <v>75</v>
       </c>
-      <c r="D13" t="s">
-        <v>76</v>
+      <c r="D13">
+        <v>37274</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="56">
-        <v>2.29</v>
+        <v>24</v>
       </c>
       <c r="B14" s="59">
-        <v>2.4340000000000002</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
         <v>75</v>
       </c>
-      <c r="D14" t="s">
-        <v>76</v>
+      <c r="D14">
+        <v>37274</v>
       </c>
       <c r="E14" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="58">
-        <v>2.1</v>
+        <v>128</v>
       </c>
       <c r="B15" s="57">
-        <v>2.4630000000000001</v>
+        <v>122.9</v>
       </c>
       <c r="C15" t="s">
         <v>75</v>
       </c>
-      <c r="D15" t="s">
-        <v>76</v>
+      <c r="D15">
+        <v>37274</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="58">
-        <v>1.41</v>
+        <v>128</v>
       </c>
       <c r="B16" s="57">
-        <v>1.623</v>
+        <v>137.80000000000001</v>
       </c>
       <c r="C16" t="s">
         <v>75</v>
       </c>
-      <c r="D16" t="s">
-        <v>76</v>
+      <c r="D16">
+        <v>37274</v>
       </c>
       <c r="E16" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="56">
-        <v>0.71899999999999997</v>
+        <v>31</v>
       </c>
       <c r="B17" s="59">
-        <v>0.83599999999999997</v>
+        <v>24.4</v>
       </c>
       <c r="C17" t="s">
         <v>75</v>
       </c>
-      <c r="D17" t="s">
-        <v>76</v>
+      <c r="D17">
+        <v>37274</v>
       </c>
       <c r="E17" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F17" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="58">
-        <v>1.65</v>
+        <v>31</v>
       </c>
       <c r="B18" s="57">
-        <v>1.794</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
         <v>75</v>
       </c>
-      <c r="D18" t="s">
-        <v>76</v>
+      <c r="D18">
+        <v>37274</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="56">
-        <v>0.73599999999999999</v>
+        <v>37</v>
       </c>
       <c r="B19" s="59">
-        <v>0.94299999999999995</v>
+        <v>38.6</v>
       </c>
       <c r="C19" t="s">
         <v>75</v>
       </c>
-      <c r="D19" t="s">
-        <v>76</v>
+      <c r="D19">
+        <v>37274</v>
       </c>
       <c r="E19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+      <c r="F19" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="58">
-        <v>1.77</v>
+        <v>37</v>
       </c>
       <c r="B20" s="57">
-        <v>2.1349999999999998</v>
+        <v>0</v>
       </c>
       <c r="C20" t="s">
         <v>75</v>
       </c>
-      <c r="D20" t="s">
-        <v>76</v>
+      <c r="D20">
+        <v>37274</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="56"/>
-      <c r="B21" s="59"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="58"/>
-      <c r="B22" s="57"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="58"/>
-      <c r="B23" s="57"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="44"/>
-      <c r="B24" s="44"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="44"/>
-      <c r="B25" s="44"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="44"/>
-      <c r="B26" s="44"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="56"/>
-      <c r="B27" s="59"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="58"/>
-      <c r="B28" s="57"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="56"/>
-      <c r="B29" s="59"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="58"/>
-      <c r="B30" s="57"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="56"/>
-      <c r="B31" s="59"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="56"/>
-      <c r="B32" s="59"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="58"/>
-      <c r="B33" s="57"/>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="56"/>
-      <c r="B34" s="59"/>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="58"/>
-      <c r="B35" s="57"/>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="56"/>
-      <c r="B36" s="59"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="58"/>
-      <c r="B37" s="57"/>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="44"/>
-      <c r="B38" s="59"/>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="58"/>
-      <c r="B39" s="59"/>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="56"/>
-      <c r="B40" s="57"/>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="58"/>
-      <c r="B41" s="59"/>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="56"/>
-      <c r="B42" s="57"/>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="58"/>
-      <c r="B43" s="59"/>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="56"/>
-      <c r="B44" s="57"/>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="56"/>
-      <c r="B45" s="57"/>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="58"/>
-      <c r="B46" s="59"/>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="56"/>
-      <c r="B47" s="57"/>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A48" s="58"/>
-      <c r="B48" s="59"/>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A49" s="56"/>
-      <c r="B49" s="57"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A21" s="56">
+        <v>117</v>
+      </c>
+      <c r="B21" s="59">
+        <v>118.4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D21">
+        <v>37274</v>
+      </c>
+      <c r="E21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="58">
+        <v>117</v>
+      </c>
+      <c r="B22" s="57">
+        <v>124</v>
+      </c>
+      <c r="C22" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22">
+        <v>37274</v>
+      </c>
+      <c r="E22" t="s">
+        <v>76</v>
+      </c>
+      <c r="F22" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" s="58">
+        <v>31</v>
+      </c>
+      <c r="B23" s="57">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="C23" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23">
+        <v>37274</v>
+      </c>
+      <c r="E23" t="s">
+        <v>76</v>
+      </c>
+      <c r="F23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="44">
+        <v>50</v>
+      </c>
+      <c r="B24" s="44">
+        <v>48.4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24">
+        <v>37274</v>
+      </c>
+      <c r="E24" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="44">
+        <v>50</v>
+      </c>
+      <c r="B25" s="44">
+        <v>52.2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>75</v>
+      </c>
+      <c r="D25">
+        <v>37274</v>
+      </c>
+      <c r="E25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F25" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="44">
+        <v>299</v>
+      </c>
+      <c r="B26" s="44">
+        <v>312</v>
+      </c>
+      <c r="C26" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26">
+        <v>37274</v>
+      </c>
+      <c r="E26" t="s">
+        <v>76</v>
+      </c>
+      <c r="F26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="56">
+        <v>1215</v>
+      </c>
+      <c r="B27" s="59">
+        <v>1174.5999999999999</v>
+      </c>
+      <c r="C27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D27">
+        <v>37274</v>
+      </c>
+      <c r="E27" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="58">
+        <v>1215</v>
+      </c>
+      <c r="B28" s="57">
+        <v>1224.4000000000001</v>
+      </c>
+      <c r="C28" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28">
+        <v>37274</v>
+      </c>
+      <c r="E28" t="s">
+        <v>76</v>
+      </c>
+      <c r="F28" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" s="56">
+        <v>9</v>
+      </c>
+      <c r="B29" s="59">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="C29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D29">
+        <v>37274</v>
+      </c>
+      <c r="E29" t="s">
+        <v>76</v>
+      </c>
+      <c r="F29" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" s="58">
+        <v>9</v>
+      </c>
+      <c r="B30" s="57">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="C30" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30">
+        <v>37274</v>
+      </c>
+      <c r="E30" t="s">
+        <v>76</v>
+      </c>
+      <c r="F30" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" s="56">
+        <v>9</v>
+      </c>
+      <c r="B31" s="59">
+        <v>9.5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31">
+        <v>37274</v>
+      </c>
+      <c r="E31" t="s">
+        <v>76</v>
+      </c>
+      <c r="F31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" s="56">
+        <v>96</v>
+      </c>
+      <c r="B32" s="59">
+        <v>96.4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D32">
+        <v>37274</v>
+      </c>
+      <c r="E32" t="s">
+        <v>76</v>
+      </c>
+      <c r="F32" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A33" s="58">
+        <v>202</v>
+      </c>
+      <c r="B33" s="57">
+        <v>193.4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33">
+        <v>37274</v>
+      </c>
+      <c r="E33" t="s">
+        <v>76</v>
+      </c>
+      <c r="F33" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" s="56">
+        <v>202</v>
+      </c>
+      <c r="B34" s="59">
+        <v>213.3</v>
+      </c>
+      <c r="C34" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34">
+        <v>37274</v>
+      </c>
+      <c r="E34" t="s">
+        <v>76</v>
+      </c>
+      <c r="F34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" s="58">
+        <v>64</v>
+      </c>
+      <c r="B35" s="57">
+        <v>58.2</v>
+      </c>
+      <c r="C35" t="s">
+        <v>75</v>
+      </c>
+      <c r="D35">
+        <v>37274</v>
+      </c>
+      <c r="E35" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A36" s="56">
+        <v>64</v>
+      </c>
+      <c r="B36" s="59">
+        <v>68.2</v>
+      </c>
+      <c r="C36" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36">
+        <v>37274</v>
+      </c>
+      <c r="E36" t="s">
+        <v>76</v>
+      </c>
+      <c r="F36" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A37" s="58">
+        <v>98</v>
+      </c>
+      <c r="B37" s="57">
+        <v>91.9</v>
+      </c>
+      <c r="C37" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37">
+        <v>37274</v>
+      </c>
+      <c r="E37" t="s">
+        <v>76</v>
+      </c>
+      <c r="F37" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A38" s="44">
+        <v>176</v>
+      </c>
+      <c r="B38" s="59">
+        <v>200.5</v>
+      </c>
+      <c r="C38" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38">
+        <v>37274</v>
+      </c>
+      <c r="E38" t="s">
+        <v>76</v>
+      </c>
+      <c r="F38" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A39" s="58">
+        <v>21</v>
+      </c>
+      <c r="B39" s="59">
+        <v>20.2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39">
+        <v>37274</v>
+      </c>
+      <c r="E39" t="s">
+        <v>76</v>
+      </c>
+      <c r="F39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A40" s="56">
+        <v>28</v>
+      </c>
+      <c r="B40" s="57">
+        <v>29.9</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40">
+        <v>37274</v>
+      </c>
+      <c r="E40" t="s">
+        <v>76</v>
+      </c>
+      <c r="F40" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A41" s="58">
+        <v>116</v>
+      </c>
+      <c r="B41" s="59">
+        <v>116.3</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41">
+        <v>37274</v>
+      </c>
+      <c r="E41" t="s">
+        <v>76</v>
+      </c>
+      <c r="F41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A42" s="56">
+        <v>18</v>
+      </c>
+      <c r="B42" s="57">
+        <v>18.3</v>
+      </c>
+      <c r="C42" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42">
+        <v>37274</v>
+      </c>
+      <c r="E42" t="s">
+        <v>76</v>
+      </c>
+      <c r="F42" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" s="58">
+        <v>382</v>
+      </c>
+      <c r="B43" s="59">
+        <v>381.4</v>
+      </c>
+      <c r="C43" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43">
+        <v>37274</v>
+      </c>
+      <c r="E43" t="s">
+        <v>76</v>
+      </c>
+      <c r="F43" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A44" s="56">
+        <v>382</v>
+      </c>
+      <c r="B44" s="57">
+        <v>448.1</v>
+      </c>
+      <c r="C44" t="s">
+        <v>75</v>
+      </c>
+      <c r="D44">
+        <v>37274</v>
+      </c>
+      <c r="E44" t="s">
+        <v>76</v>
+      </c>
+      <c r="F44" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A45" s="56">
+        <v>48</v>
+      </c>
+      <c r="B45" s="57">
+        <v>48.6</v>
+      </c>
+      <c r="C45" t="s">
+        <v>75</v>
+      </c>
+      <c r="D45">
+        <v>37274</v>
+      </c>
+      <c r="E45" t="s">
+        <v>76</v>
+      </c>
+      <c r="F45" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" s="58">
+        <v>115</v>
+      </c>
+      <c r="B46" s="59">
+        <v>126.5</v>
+      </c>
+      <c r="C46" t="s">
+        <v>75</v>
+      </c>
+      <c r="D46">
+        <v>37274</v>
+      </c>
+      <c r="E46" t="s">
+        <v>76</v>
+      </c>
+      <c r="F46" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A47" s="56">
+        <v>14</v>
+      </c>
+      <c r="B47" s="57">
+        <v>15.5</v>
+      </c>
+      <c r="C47" t="s">
+        <v>75</v>
+      </c>
+      <c r="D47">
+        <v>37274</v>
+      </c>
+      <c r="E47" t="s">
+        <v>76</v>
+      </c>
+      <c r="F47" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A48" s="58">
+        <v>210</v>
+      </c>
+      <c r="B48" s="59">
+        <v>194.9</v>
+      </c>
+      <c r="C48" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48">
+        <v>37274</v>
+      </c>
+      <c r="E48" t="s">
+        <v>76</v>
+      </c>
+      <c r="F48" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A49" s="56">
+        <v>22</v>
+      </c>
+      <c r="B49" s="57">
+        <v>21.9</v>
+      </c>
+      <c r="C49" t="s">
+        <v>75</v>
+      </c>
+      <c r="D49">
+        <v>37274</v>
+      </c>
+      <c r="E49" t="s">
+        <v>76</v>
+      </c>
+      <c r="F49" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="58"/>
       <c r="B50" s="59"/>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="56"/>
       <c r="B51" s="57"/>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="58"/>
       <c r="B52" s="59"/>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="56"/>
       <c r="B53" s="57"/>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="58"/>
       <c r="B54" s="59"/>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="56"/>
       <c r="B55" s="57"/>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="58"/>
       <c r="B56" s="59"/>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="56"/>
       <c r="B57" s="57"/>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="58"/>
       <c r="B58" s="59"/>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="56"/>
       <c r="B59" s="57"/>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="58"/>
       <c r="B60" s="59"/>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="56"/>
       <c r="B61" s="57"/>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="58"/>
       <c r="B62" s="59"/>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="56"/>
       <c r="B63" s="57"/>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="58"/>
       <c r="B64" s="59"/>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="56"/>
       <c r="B65" s="57"/>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="58"/>
       <c r="B66" s="59"/>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="56"/>
       <c r="B67" s="57"/>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="58"/>
       <c r="B68" s="59"/>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="56"/>
       <c r="B69" s="57"/>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="58"/>
       <c r="B70" s="59"/>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="56"/>
       <c r="B71" s="57"/>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="58"/>
       <c r="B72" s="59"/>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="56"/>
       <c r="B73" s="57"/>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" s="58"/>
       <c r="B74" s="59"/>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" s="56"/>
       <c r="B75" s="57"/>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" s="58"/>
       <c r="B76" s="59"/>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" s="56"/>
       <c r="B77" s="57"/>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" s="58"/>
       <c r="B78" s="59"/>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" s="56"/>
       <c r="B79" s="57"/>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" s="58"/>
       <c r="B80" s="59"/>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" s="56"/>
       <c r="B81" s="57"/>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" s="58"/>
       <c r="B82" s="59"/>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" s="56"/>
       <c r="B83" s="57"/>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" s="58"/>
       <c r="B84" s="59"/>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" s="56"/>
       <c r="B85" s="57"/>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" s="58"/>
       <c r="B86" s="59"/>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" s="56"/>
       <c r="B87" s="57"/>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" s="58"/>
       <c r="B88" s="59"/>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" s="56"/>
       <c r="B89" s="57"/>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" s="58"/>
       <c r="B90" s="59"/>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" s="56"/>
       <c r="B91" s="57"/>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" s="58"/>
       <c r="B92" s="59"/>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" s="56"/>
       <c r="B93" s="57"/>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" s="58"/>
       <c r="B94" s="59"/>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" s="56"/>
       <c r="B95" s="57"/>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" s="58"/>
       <c r="B96" s="59"/>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" s="56"/>
       <c r="B97" s="57"/>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" s="58"/>
       <c r="B98" s="59"/>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" s="56"/>
       <c r="B99" s="57"/>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" s="58"/>
       <c r="B100" s="59"/>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" s="56"/>
       <c r="B101" s="57"/>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" s="58"/>
       <c r="B102" s="59"/>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" s="56"/>
       <c r="B103" s="57"/>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" s="58"/>
       <c r="B104" s="59"/>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" s="56"/>
       <c r="B105" s="57"/>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" s="58"/>
       <c r="B106" s="59"/>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" s="56"/>
       <c r="B107" s="57"/>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" s="58"/>
       <c r="B108" s="59"/>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" s="56"/>
       <c r="B109" s="57"/>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" s="58"/>
       <c r="B110" s="59"/>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" s="56"/>
       <c r="B111" s="57"/>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" s="58"/>
       <c r="B112" s="59"/>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" s="56"/>
       <c r="B113" s="57"/>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" s="58"/>
       <c r="B114" s="59"/>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" s="56"/>
       <c r="B115" s="57"/>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" s="58"/>
       <c r="B116" s="59"/>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" s="56"/>
       <c r="B117" s="57"/>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" s="58"/>
       <c r="B118" s="59"/>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" s="56"/>
       <c r="B119" s="57"/>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" s="58"/>
       <c r="B120" s="59"/>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" s="56"/>
       <c r="B121" s="57"/>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" s="58"/>
       <c r="B122" s="59"/>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" s="56"/>
       <c r="B123" s="57"/>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" s="58"/>
       <c r="B124" s="59"/>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" s="56"/>
       <c r="B125" s="57"/>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" s="58"/>
       <c r="B126" s="59"/>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" s="56"/>
       <c r="B127" s="57"/>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" s="58"/>
       <c r="B128" s="59"/>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" s="56"/>
       <c r="B129" s="57"/>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" s="58"/>
       <c r="B130" s="59"/>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" s="56"/>
       <c r="B131" s="57"/>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" s="58"/>
       <c r="B132" s="59"/>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" s="56"/>
       <c r="B133" s="57"/>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" s="58"/>
       <c r="B134" s="59"/>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" s="56"/>
       <c r="B135" s="57"/>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" s="58"/>
       <c r="B136" s="59"/>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" s="56"/>
       <c r="B137" s="57"/>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" s="58"/>
       <c r="B138" s="59"/>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" s="56"/>
       <c r="B139" s="57"/>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" s="58"/>
       <c r="B140" s="59"/>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A141" s="56"/>
       <c r="B141" s="57"/>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A142" s="58"/>
       <c r="B142" s="59"/>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A143" s="56"/>
       <c r="B143" s="57"/>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A144" s="58"/>
       <c r="B144" s="59"/>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A145" s="56"/>
       <c r="B145" s="57"/>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A146" s="58"/>
       <c r="B146" s="59"/>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A147" s="56"/>
       <c r="B147" s="57"/>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A148" s="60"/>
       <c r="B148" s="55"/>
     </row>

</xml_diff>